<commit_message>
feat(exhibits): finalize Model A reorganization and redirect figure workbooks via Method 1
</commit_message>
<xml_diff>
--- a/thesis_docs/exhibits/ch03_methodology/workbooks/01_Sample_and_Airport_Selection.xlsx
+++ b/thesis_docs/exhibits/ch03_methodology/workbooks/01_Sample_and_Airport_Selection.xlsx
@@ -546,7 +546,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
@@ -869,7 +869,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
@@ -1084,7 +1084,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -1246,7 +1246,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -1554,7 +1554,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -1738,7 +1738,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -1944,7 +1944,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
@@ -2114,7 +2114,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>

</xml_diff>